<commit_message>
Adding javadoc style comments and updating README accordingly
</commit_message>
<xml_diff>
--- a/data/S.aureus/Howden2023_S.aureus_virulence-factor-list.xlsx
+++ b/data/S.aureus/Howden2023_S.aureus_virulence-factor-list.xlsx
@@ -532,7 +532,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -573,7 +573,7 @@
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general" wrapText="1"/>
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1142,7 +1142,7 @@
         <v>66</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="60" customFormat="1" s="1">
       <c r="A16" s="2" t="s">
         <v>67</v>
       </c>
@@ -1159,7 +1159,7 @@
         <v>71</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="19.5" customFormat="1" s="1">
       <c r="A17" s="2" t="s">
         <v>72</v>
       </c>
@@ -1176,7 +1176,7 @@
         <v>76</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="73.5" customFormat="1" s="1">
       <c r="A18" s="2" t="s">
         <v>77</v>
       </c>
@@ -1193,7 +1193,7 @@
         <v>80</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="19.5" customFormat="1" s="1">
       <c r="A19" s="2" t="s">
         <v>81</v>
       </c>
@@ -1210,7 +1210,7 @@
         <v>24</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="46.5" customFormat="1" s="1">
       <c r="A20" s="2" t="s">
         <v>84</v>
       </c>
@@ -1227,7 +1227,7 @@
         <v>88</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="46.5" customFormat="1" s="1">
       <c r="A21" s="2" t="s">
         <v>89</v>
       </c>
@@ -1244,7 +1244,7 @@
         <v>93</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="19.5" customFormat="1" s="1">
       <c r="A22" s="2" t="s">
         <v>94</v>
       </c>
@@ -1261,7 +1261,7 @@
         <v>97</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="60" customFormat="1" s="1">
       <c r="A23" s="2" t="s">
         <v>98</v>
       </c>
@@ -1278,7 +1278,7 @@
         <v>102</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="19.5" customFormat="1" s="1">
       <c r="A24" s="2" t="s">
         <v>103</v>
       </c>
@@ -1295,7 +1295,7 @@
         <v>97</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="33" customFormat="1" s="1">
       <c r="A25" s="2" t="s">
         <v>107</v>
       </c>
@@ -1312,7 +1312,7 @@
         <v>111</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18.75" customFormat="1" s="1">
+    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="33" customFormat="1" s="1">
       <c r="A26" s="2" t="s">
         <v>112</v>
       </c>

</xml_diff>